<commit_message>
feat: add compare tab, tie-breaker precision, and utility scripts
</commit_message>
<xml_diff>
--- a/outputs/submission.xlsx
+++ b/outputs/submission.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.824745</v>
+        <v>0.838303</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -466,7 +466,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.807396</v>
+        <v>0.82556</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.802227</v>
+        <v>0.812275</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.781293</v>
+        <v>0.803558</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.765279</v>
+        <v>0.782097</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -531,36 +531,36 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.757265</v>
+        <v>0.782038</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.5 yrs, currently NLP Engineer at Haptik -- career history shows embeddings/retrieval work; based in Pune, Maharashtra; 15-day notice.</t>
+          <t>Recommendation Systems Engineer at CRED (8.0 yrs); career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; 77% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.755734</v>
+        <v>0.77381</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at CRED (8.0 yrs); career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; 77% recruiter response rate.</t>
+          <t>6.5 yrs, currently NLP Engineer at Haptik -- career history shows embeddings/retrieval work; based in Pune, Maharashtra; 15-day notice.</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.734897</v>
+        <v>0.764462</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.726351</v>
+        <v>0.74951</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -603,36 +603,36 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.71468</v>
+        <v>0.727429</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6.8 yrs, currently AI Engineer at Rephrase.ai -- career history shows embeddings/retrieval work; based in Delhi, Delhi; 77% recruiter response rate; 30-day notice.</t>
+          <t>6.9 yrs as AI Engineer at Microsoft; career history shows embeddings/retrieval work; based in Trivandrum, Kerala; 81% recruiter response rate; 30-day notice.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.711587</v>
+        <v>0.725895</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.9 yrs as AI Engineer at Microsoft; career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>AI Engineer at Rephrase.ai, 6.8 yrs. career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.687001</v>
+        <v>0.705417</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.665179</v>
+        <v>0.686752</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -675,36 +675,36 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.664737</v>
+        <v>0.677821</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.3 yrs as AI Engineer at Google; career history shows embeddings/retrieval work; based in Kochi, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Applied ML Engineer at Meta, 4.7 yrs. career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.658027</v>
+        <v>0.674222</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Meta, 4.7 yrs. career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>7.3 yrs as AI Engineer at Google; career history shows embeddings/retrieval work; based in Kochi, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.655408</v>
+        <v>0.658074</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.646497</v>
+        <v>0.648509</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.641639</v>
+        <v>0.646864</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.624021</v>
+        <v>0.639036</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -783,72 +783,72 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.621124</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at BYJU'S, 4.5 yrs. career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>6.6 yrs as Applied ML Engineer at Sarvam AI; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: long notice period (90 days).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.620671</v>
+        <v>0.632173</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>6.6 yrs as Applied ML Engineer at Sarvam AI; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: long notice period (90 days).</t>
+          <t>Senior AI Engineer at Netflix, 7.8 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.613596</v>
+        <v>0.631515</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Netflix, 7.8 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Machine Learning Engineer at BYJU'S, 4.5 yrs. career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.613297</v>
+        <v>0.6300789999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Mad Street Den, 5.9 yrs. career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>5.2 yrs as Senior NLP Engineer at Netflix; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.610993</v>
+        <v>0.626794</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -873,90 +873,90 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.610776</v>
+        <v>0.626059</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.2 yrs as Senior NLP Engineer at Netflix; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Senior Data Scientist at Mad Street Den, 5.9 yrs. career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.605997</v>
+        <v>0.625658</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Niramai, 7.8 yrs. career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>NLP Engineer at Aganitha, 6.6 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.605392</v>
+        <v>0.623452</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Search Engineer at Nykaa, 7.8 yrs. career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Senior NLP Engineer at Niramai, 7.8 yrs. career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.605108</v>
+        <v>0.622845</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NLP Engineer at Aganitha, 6.6 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>8.8 yrs as Staff Machine Learning Engineer at Salesforce; career history shows embeddings/retrieval work; based in Coimbatore, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.601214</v>
+        <v>0.619111</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>8.8 yrs as Staff Machine Learning Engineer at Salesforce; career history shows embeddings/retrieval work; based in Coimbatore, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>5.3 yrs as Senior Applied Scientist at Sarvam AI; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.596247</v>
+        <v>0.614877</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -981,270 +981,270 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.594982</v>
+        <v>0.614861</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AI Engineer at PolicyBazaar, 7.7 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>7.7 yrs as Recommendation Systems Engineer at Nykaa; career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5920029999999999</v>
+        <v>0.611047</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5.2 yrs as Senior Data Scientist at Niramai; career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days).</t>
+          <t>Search Engineer at Nykaa, 7.8 yrs. career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.590815</v>
+        <v>0.609439</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Zoho, 6.6 yrs. career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: long notice period (120 days).</t>
+          <t>Recommendation Systems Engineer at CRED, 6.0 yrs. career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.590476</v>
+        <v>0.606077</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at CRED, 6.0 yrs. career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Machine Learning Engineer at Haptik, 5.7 yrs. career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.590452</v>
+        <v>0.605284</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5.3 yrs as Senior Applied Scientist at Sarvam AI; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Recommendation Systems Engineer at Zoho, 6.6 yrs. career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: long notice period (120 days).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.589854</v>
+        <v>0.603508</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>7.7 yrs as Recommendation Systems Engineer at Nykaa; career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>5.1 yrs as Applied ML Engineer at CRED; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.5879799999999999</v>
+        <v>0.601056</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Haptik, 5.7 yrs. career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>AI Engineer at PolicyBazaar, 7.7 yrs. career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.586094</v>
+        <v>0.600872</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5.1 yrs as Applied ML Engineer at CRED; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Search Engineer at Verloop.io, 4.2 yrs. career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.585508</v>
+        <v>0.596886</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Search Engineer at Verloop.io, 4.2 yrs. career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>5.2 yrs as Senior Data Scientist at Niramai; career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.577993</v>
+        <v>0.594278</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Razorpay, 5.3 yrs. career history shows embeddings/retrieval work; based in Chandigarh, Chandigarh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Senior AI Engineer at Apple, 5.9 yrs. career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0075249</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.57784</v>
+        <v>0.590829</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Apple, 5.9 yrs. career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Applied ML Engineer at Zomato, 6.2 yrs. career history shows embeddings/retrieval work; based in Ahmedabad, Gujarat; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0076251</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.571535</v>
+        <v>0.583704</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>7.6 yrs as Search Engineer at Haptik; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>6.7 yrs as NLP Engineer at Rephrase.ai; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0075249</t>
+          <t>CAND_0054394</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5684</v>
+        <v>0.583472</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Zomato, 6.2 yrs. career history shows embeddings/retrieval work; based in Ahmedabad, Gujarat; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>4.1 yrs as Recommendation Systems Engineer at PharmEasy; career history shows embeddings/retrieval work; based in Pune, Maharashtra; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.564068</v>
+        <v>0.579597</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6.7 yrs as NLP Engineer at Rephrase.ai; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>7.6 yrs as Search Engineer at Haptik; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0054394</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.563621</v>
+        <v>0.578202</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>4.1 yrs as Recommendation Systems Engineer at PharmEasy; career history shows embeddings/retrieval work; based in Pune, Maharashtra; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Senior Data Scientist at Razorpay, 5.3 yrs. career history shows embeddings/retrieval work; based in Chandigarh, Chandigarh; concern: strong embeddings/retrieval experience in career history.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.562932</v>
+        <v>0.577755</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1269,72 +1269,72 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0066376</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.553152</v>
+        <v>0.574166</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Dream11, 5.7 yrs. career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: long notice period (90 days).</t>
+          <t>Applied ML Engineer at Meesho, 7.1 yrs. career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: long notice period (90 days).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.551855</v>
+        <v>0.572078</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Meesho, 7.1 yrs. career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: long notice period (90 days).</t>
+          <t>Applied ML Engineer at Dream11, 6.7 yrs. career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: long notice period (120 days).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0066376</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.551755</v>
+        <v>0.571637</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>6.5 yrs as Senior Data Scientist at Google; career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days).</t>
+          <t>Applied ML Engineer at Dream11, 5.7 yrs. career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: long notice period (90 days).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0098846</t>
+          <t>CAND_0007412</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.547673</v>
+        <v>0.569424</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>7.6 yrs as AI Engineer at upGrad; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history.</t>
+          <t>Applied ML Engineer at Zoho, 7.4 yrs. career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days).</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.546521</v>
+        <v>0.567089</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1359,378 +1359,378 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.546333</v>
+        <v>0.565044</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>6.8 yrs as Applied ML Engineer at Zoho; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Recommendation Systems Engineer at Swiggy (6.0 yrs). career history shows embeddings/retrieval work; based in Hyderabad, Telangana; concern: has ranking-evaluation framework experience; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.546195</v>
+        <v>0.565004</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>7.2 yrs as Search Engineer at Google; career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.8 yrs as Applied ML Engineer at Zoho; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.545697</v>
+        <v>0.563114</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>8.6 yrs as Lead AI Engineer at Meta; career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.5 yrs as Senior Data Scientist at Google; career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0007412</t>
+          <t>CAND_0053695</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.544924</v>
+        <v>0.55788</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Zoho (7.4 yrs). career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: long notice period (120 days); weaker fit than the candidates above.</t>
+          <t>5.8 yrs as Recommendation Systems Engineer at Meesho; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.543743</v>
+        <v>0.557482</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>4.7 yrs as Senior Data Scientist at CRED; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Machine Learning Engineer at Genpact AI (7.2 yrs). career history shows embeddings/retrieval work; based in Kochi, Kerala; concern: long notice period (120 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0098846</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.542483</v>
+        <v>0.557482</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Dream11 (6.7 yrs). career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: long notice period (120 days); weaker fit than the candidates above.</t>
+          <t>7.6 yrs as AI Engineer at upGrad; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.542441</v>
+        <v>0.552777</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Genpact AI (7.2 yrs). career history shows embeddings/retrieval work; based in Kochi, Kerala; concern: long notice period (120 days); weaker fit than the candidates above.</t>
+          <t>4.7 yrs as Senior Data Scientist at CRED; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.540837</v>
+        <v>0.552583</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Swiggy (6.0 yrs). career history shows embeddings/retrieval work; based in Hyderabad, Telangana; concern: has ranking-evaluation framework experience; weaker fit than the candidates above.</t>
+          <t>7.2 yrs as Search Engineer at Google; career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.5396300000000001</v>
+        <v>0.547894</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Search Engineer at CRED (7.8 yrs). career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (120 days); weaker fit than the candidates above.</t>
+          <t>8.6 yrs as Lead AI Engineer at Meta; career history shows embeddings/retrieval work; based in Mumbai, Maharashtra; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0053695</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.537537</v>
+        <v>0.547494</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>5.8 yrs as Recommendation Systems Engineer at Meesho; career history shows embeddings/retrieval work; based in Bhubaneswar, Odisha; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Search Engineer at CRED (7.8 yrs). career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (120 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.536727</v>
+        <v>0.54609</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Ola (7.8 yrs). career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>8.1 yrs as Senior Machine Learning Engineer at Flipkart; career history shows embeddings/retrieval work; based in London; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.53084</v>
+        <v>0.543788</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>8.1 yrs as Senior Machine Learning Engineer at Flipkart; career history shows embeddings/retrieval work; based in London; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>NLP Engineer at Krutrim (5.2 yrs). career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.529543</v>
+        <v>0.539104</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>NLP Engineer at Krutrim (5.2 yrs). career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
+          <t>5.7 yrs as Machine Learning Engineer at Verloop.io; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: has ranking-evaluation framework experience -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0003977</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.528073</v>
+        <v>0.538707</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Google (4.6 yrs). career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
+          <t>Applied ML Engineer at Freshworks (5.2 yrs). career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.521992</v>
+        <v>0.538697</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Freshworks (5.2 yrs). career history shows embeddings/retrieval work; based in Trivandrum, Kerala; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
+          <t>Senior NLP Engineer at Ola (7.8 yrs). career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.5204299999999999</v>
+        <v>0.538026</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>7.2 yrs as AI Engineer at Vedantu; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.5 yrs as Recommendation Systems Engineer at PhonePe; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.519876</v>
+        <v>0.5373559999999999</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>5.7 yrs as Machine Learning Engineer at Verloop.io; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: has ranking-evaluation framework experience -- a lower-confidence fit included to round out the top 100.</t>
+          <t>7.2 yrs as AI Engineer at Vedantu; career history shows embeddings/retrieval work; based in Gurgaon, Haryana; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.514413</v>
+        <v>0.537201</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>6.5 yrs as Recommendation Systems Engineer at PhonePe; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.9 yrs as Machine Learning Engineer at LinkedIn; career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0003977</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.514095</v>
+        <v>0.53699</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6.9 yrs as Machine Learning Engineer at LinkedIn; career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Recommendation Systems Engineer at Google (4.6 yrs). career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0086151</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.513655</v>
+        <v>0.528528</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>7.7 yrs as Recommendation Systems Engineer at Wysa; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.4 yrs as Lead AI Engineer at Sarvam AI; career history shows vector DB/hybrid search work; based in Delhi, Delhi; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0058575</t>
+          <t>CAND_0086151</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.513198</v>
+        <v>0.528315</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>AI Engineer at Krutrim (5.8 yrs). career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>7.7 yrs as Recommendation Systems Engineer at Wysa; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.508169</v>
+        <v>0.527824</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1755,72 +1755,72 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.505796</v>
+        <v>0.5260359999999999</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Rephrase.ai (5.7 yrs). career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>Senior AI Engineer at Meta (7.9 yrs). career history shows ranking evaluation (NDCG/MRR/MAP) work; based in Noida, Uttar Pradesh; concern: little/no production embeddings-retrieval evidence; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.502238</v>
+        <v>0.525458</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Nykaa (5.5 yrs). career history shows embeddings/retrieval work; based in Ahmedabad, Gujarat; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
+          <t>8.0 yrs as Staff Machine Learning Engineer at LinkedIn; career history shows ranking evaluation (NDCG/MRR/MAP) work; based in Noida, Uttar Pradesh; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0008295</t>
+          <t>CAND_0058575</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.501961</v>
+        <v>0.525107</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>6.5 yrs as AI Research Engineer at Razorpay; career history shows vector DB/hybrid search work; based in Pune, Maharashtra; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
+          <t>AI Engineer at Krutrim (5.8 yrs). career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.5015849999999999</v>
+        <v>0.520647</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>6.4 yrs as Lead AI Engineer at Sarvam AI; career history shows vector DB/hybrid search work; based in Delhi, Delhi; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Recommendation Systems Engineer at Nykaa (5.5 yrs). career history shows embeddings/retrieval work; based in Ahmedabad, Gujarat; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.499099</v>
+        <v>0.51117</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1845,54 +1845,54 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0031593</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.49903</v>
+        <v>0.510672</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Search Engineer at Genpact AI (7.8 yrs). career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 yrs). career history shows embeddings/retrieval work; based in Jaipur, Rajasthan; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0031593</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.497781</v>
+        <v>0.5097660000000001</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Meta (7.9 yrs). career history shows ranking evaluation (NDCG/MRR/MAP) work; based in Noida, Uttar Pradesh; concern: little/no production embeddings-retrieval evidence; weaker fit than the candidates above.</t>
+          <t>Search Engineer at Genpact AI (7.8 yrs). career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.495213</v>
+        <v>0.509161</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>8.0 yrs as Staff Machine Learning Engineer at LinkedIn; career history shows ranking evaluation (NDCG/MRR/MAP) work; based in Noida, Uttar Pradesh; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Senior Data Scientist at Rephrase.ai (5.7 yrs). career history shows embeddings/retrieval work; based in Bangalore, Karnataka; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.493573</v>
+        <v>0.504542</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -1917,162 +1917,162 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.492923</v>
+        <v>0.50321</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 yrs). career history shows embeddings/retrieval work; based in Jaipur, Rajasthan; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>5.3 yrs as Senior Data Scientist at Netflix; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0020708</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.492524</v>
+        <v>0.501096</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>5.3 yrs as Senior Data Scientist at Netflix; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Search Engineer at PolicyBazaar (4.2 yrs). career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0020708</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.49096</v>
+        <v>0.498959</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Search Engineer at PolicyBazaar (4.2 yrs). career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history; weaker fit than the candidates above.</t>
+          <t>5.4 yrs as AI Engineer at Zoho; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.48738</v>
+        <v>0.497556</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>5.4 yrs as AI Engineer at Zoho; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>7.3 yrs as Search Engineer at Unacademy; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0052335</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.485525</v>
+        <v>0.496241</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>7.6 yrs as Senior Data Scientist at Amazon; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.4 yrs as Applied ML Engineer at Aganitha; career history shows embeddings/retrieval work; based in Berlin; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.485209</v>
+        <v>0.494005</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>7.3 yrs as Search Engineer at Unacademy; career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>7.6 yrs as Senior Data Scientist at Amazon; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.482346</v>
+        <v>0.492573</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>5.4 yrs as Senior Software Engineer (ML) at Mad Street Den; career history shows embeddings/retrieval work; based in Hyderabad, Telangana; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Recommendation Systems Engineer at Saarthi.ai (6.6 yrs). career history shows embeddings/retrieval work; based in Toronto; concern: long notice period (90 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.482134</v>
+        <v>0.492443</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Saarthi.ai (6.6 yrs). career history shows embeddings/retrieval work; based in Toronto; concern: long notice period (90 days); weaker fit than the candidates above.</t>
+          <t>NLP Engineer at Ola (6.9 yrs). career history shows embeddings/retrieval work; based in Chandigarh, Chandigarh; weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.480363</v>
+        <v>0.492</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>5.1 yrs as Search Engineer at CRED; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>Applied ML Engineer at upGrad (5.0 yrs). career history shows embeddings/retrieval work; based in Hyderabad, Telangana; concern: long notice period (120 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.480253</v>
+        <v>0.491703</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2097,144 +2097,144 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.476627</v>
+        <v>0.4912</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>16.2 yrs as Senior Applied Scientist at Meta; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>6.0 yrs as Applied ML Engineer at Freshworks; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0094056</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.47598</v>
+        <v>0.490687</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>5.9 yrs as NLP Engineer at Rephrase.ai; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>5.1 yrs as Search Engineer at CRED; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0052335</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.473792</v>
+        <v>0.487923</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>6.4 yrs as Applied ML Engineer at Aganitha; career history shows embeddings/retrieval work; based in Berlin; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>16.2 yrs as Senior Applied Scientist at Meta; career history shows embeddings/retrieval work; based in Indore, Madhya Pradesh; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0074225</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.473174</v>
+        <v>0.487585</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) at Tech Mahindra (6.4 yrs). career history shows embeddings/retrieval work; based in Noida, Uttar Pradesh; concern: little/no production embeddings-retrieval evidence; weaker fit than the candidates above.</t>
+          <t>Machine Learning Engineer at Unacademy (4.3 yrs). career history shows embeddings/retrieval work; based in Vizag, Andhra Pradesh; concern: long notice period (120 days); weaker fit than the candidates above.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.472349</v>
+        <v>0.487444</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>NLP Engineer at Ola (6.9 yrs). career history shows embeddings/retrieval work; based in Chandigarh, Chandigarh; weaker fit than the candidates above.</t>
+          <t>4.9 yrs as Machine Learning Engineer at Google; career history shows embeddings/retrieval work; based in Hyderabad, Telangana; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0094056</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.471844</v>
+        <v>0.487335</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>4.9 yrs as Senior Data Scientist at Vedantu; career history shows embeddings/retrieval work; based in Jaipur, Rajasthan; concern: strong embeddings/retrieval experience in career history -- a lower-confidence fit included to round out the top 100.</t>
+          <t>5.9 yrs as NLP Engineer at Rephrase.ai; career history shows embeddings/retrieval work; based in Chennai, Tamil Nadu; concern: long notice period (120 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0004402</t>
+          <t>CAND_0066999</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.471806</v>
+        <v>0.485973</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>6.0 yrs as AI Research Engineer at Yellow.ai; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
+          <t>5.9 yrs as Recommendation Systems Engineer at Microsoft; career history shows embeddings/retrieval work; based in Delhi, Delhi; concern: little/no production embeddings-retrieval evidence -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.471718</v>
+        <v>0.474187</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.0 yrs as Applied ML Engineer at Freshworks; career history shows embeddings/retrieval work; based in Kolkata, West Bengal; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
+          <t>7.7 yrs as NLP Engineer at Dream11; career history shows embeddings/retrieval work; based in Ahmedabad, Gujarat; concern: long notice period (90 days) -- a lower-confidence fit included to round out the top 100.</t>
         </is>
       </c>
     </row>

</xml_diff>